<commit_message>
Daily EOD data and reports for 2026-10-26
</commit_message>
<xml_diff>
--- a/asx_eod_output/Report_XLSX/Report_20261026.xlsx
+++ b/asx_eod_output/Report_XLSX/Report_20261026.xlsx
@@ -488,24 +488,24 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>1.49</v>
+        <v>1.44</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.015</v>
+        <v>-0.035</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.02%</t>
+          <t>-2.37%</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
         <v>153181</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>228239.69</v>
+        <v>220580.64</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>2297.71</v>
+        <v>-5361.34</v>
       </c>
     </row>
     <row r="5">
@@ -515,24 +515,24 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2.41</v>
+        <v>2.45</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0</v>
+        <v>0.04</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>1.66%</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>70000</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>168700</v>
+        <v>171500</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>0</v>
+        <v>2800</v>
       </c>
     </row>
     <row r="6">
@@ -542,24 +542,24 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>55.77</v>
+        <v>55.62</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.72</v>
+        <v>0.57</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.31%</t>
+          <t>1.04%</t>
         </is>
       </c>
       <c r="E6" s="3" t="n">
         <v>8000</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>446160</v>
+        <v>444960</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>5760</v>
+        <v>4560</v>
       </c>
     </row>
     <row r="7">
@@ -596,14 +596,14 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>160.8</v>
+        <v>163.2</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>-3.2</v>
+        <v>-0.8</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-1.95%</t>
+          <t>-0.49%</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
@@ -623,24 +623,24 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>0.775</v>
+        <v>0.77</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>0.025</v>
+        <v>0.02</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.33%</t>
+          <t>2.67%</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
         <v>10000</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>7750</v>
+        <v>7700</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>250</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -650,24 +650,24 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>191.67</v>
+        <v>195.14</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>-5.03</v>
+        <v>-1.56</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>-0.79%</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>4000</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>766680</v>
+        <v>780560</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>-20120</v>
+        <v>-6240</v>
       </c>
     </row>
     <row r="11">
@@ -677,24 +677,24 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>0.205</v>
+        <v>0.215</v>
       </c>
       <c r="C11" s="2" t="n">
-        <v>-0.005</v>
+        <v>0.005</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-2.38%</t>
+          <t>2.38%</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
         <v>20000</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4100</v>
+        <v>4300</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>-100</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12">
@@ -704,24 +704,24 @@
         </is>
       </c>
       <c r="B12" s="2" t="n">
-        <v>10.78</v>
+        <v>10.75</v>
       </c>
       <c r="C12" s="2" t="n">
-        <v>0.05</v>
+        <v>0.02</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.47%</t>
+          <t>0.19%</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
         <v>3045</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>32825.1</v>
+        <v>32733.75</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>152.25</v>
+        <v>60.9</v>
       </c>
     </row>
     <row r="13">
@@ -758,24 +758,24 @@
         </is>
       </c>
       <c r="B14" s="2" t="n">
-        <v>0.081</v>
+        <v>0.083</v>
       </c>
       <c r="C14" s="2" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>6.58%</t>
+          <t>9.21%</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
         <v>9412</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>762.37</v>
+        <v>781.2</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>47.06</v>
+        <v>65.88</v>
       </c>
     </row>
     <row r="15">
@@ -785,24 +785,24 @@
         </is>
       </c>
       <c r="B15" s="2" t="n">
-        <v>0</v>
+        <v>0.081</v>
       </c>
       <c r="C15" s="2" t="n">
-        <v>-0.08</v>
+        <v>0.001</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>-100.00%</t>
+          <t>1.25%</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
         <v>6000</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>0</v>
+        <v>486</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>-480</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
@@ -812,14 +812,14 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>36.06</v>
+        <v>36.53</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>-0.73</v>
+        <v>-0.26</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>-1.98%</t>
+          <t>-0.71%</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
@@ -839,24 +839,24 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>33.245</v>
+        <v>33.09</v>
       </c>
       <c r="C17" s="2" t="n">
-        <v>0.385</v>
+        <v>0.23</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.17%</t>
+          <t>0.70%</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
         <v>1288</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>42819.56</v>
+        <v>42619.92</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>495.88</v>
+        <v>296.24</v>
       </c>
     </row>
     <row r="18">
@@ -870,10 +870,10 @@
       <c r="D18" s="5" t="inlineStr"/>
       <c r="E18" s="7" t="inlineStr"/>
       <c r="F18" s="8" t="n">
-        <v>1698257.17</v>
+        <v>1706441.96</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>-13097.09</v>
+        <v>-4912.31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>